<commit_message>
Accomodate for different cooling sides
</commit_message>
<xml_diff>
--- a/Switch Functions/GaN Data Multitrack.xlsx
+++ b/Switch Functions/GaN Data Multitrack.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\MIT\Project\GE Vernova\Github\Switch Functions\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3660F25D-0D5D-403E-A883-1C4303E7C917}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{69160CAB-4F93-4FFE-9FA8-9CE36CF94E9A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="26">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="27">
   <si>
     <t>Part Number</t>
   </si>
@@ -47,9 +47,6 @@
     <t>Rth,JC [°C/W]</t>
   </si>
   <si>
-    <t>Coss @ Vds = 420V [pF]</t>
-  </si>
-  <si>
     <t>Lmin [mm]</t>
   </si>
   <si>
@@ -110,10 +107,16 @@
     <t>NV6029</t>
   </si>
   <si>
-    <t>Qoss @ Vds=400V [nC]</t>
-  </si>
-  <si>
     <t>Eoss @ Vds = 400V [uJ]</t>
+  </si>
+  <si>
+    <t>Coss [pF]</t>
+  </si>
+  <si>
+    <t>Cooling Side</t>
+  </si>
+  <si>
+    <t>Bottom</t>
   </si>
 </sst>
 </file>
@@ -546,7 +549,7 @@
     <col min="4" max="4" width="12.7265625" customWidth="1"/>
     <col min="5" max="5" width="20.81640625" customWidth="1"/>
     <col min="6" max="6" width="20.6328125" customWidth="1"/>
-    <col min="7" max="7" width="21.54296875" customWidth="1"/>
+    <col min="7" max="7" width="14.7265625" customWidth="1"/>
     <col min="8" max="8" width="11.6328125" customWidth="1"/>
     <col min="9" max="9" width="13.08984375" customWidth="1"/>
     <col min="10" max="10" width="13.81640625" customWidth="1"/>
@@ -559,7 +562,7 @@
   <sheetData>
     <row r="1" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A1" s="3" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B1" s="3" t="s">
         <v>0</v>
@@ -571,72 +574,72 @@
         <v>2</v>
       </c>
       <c r="E1" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="F1" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="G1" s="3" t="s">
         <v>24</v>
       </c>
-      <c r="F1" s="3" t="s">
-        <v>25</v>
-      </c>
-      <c r="G1" s="3" t="s">
+      <c r="H1" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="H1" s="5" t="s">
+      <c r="I1" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="I1" s="3" t="s">
+      <c r="J1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="K1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="L1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="M1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="M1" s="1" t="s">
-        <v>9</v>
-      </c>
       <c r="N1" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="O1" s="8" t="s">
         <v>11</v>
       </c>
-      <c r="O1" s="8" t="s">
+      <c r="P1" s="9" t="s">
         <v>12</v>
       </c>
-      <c r="P1" s="9" t="s">
+      <c r="Q1" s="9" t="s">
         <v>13</v>
       </c>
-      <c r="Q1" s="9" t="s">
+      <c r="R1" s="9" t="s">
         <v>14</v>
       </c>
-      <c r="R1" s="9" t="s">
+      <c r="S1" s="9" t="s">
         <v>15</v>
       </c>
-      <c r="S1" s="9" t="s">
+      <c r="T1" s="9" t="s">
         <v>16</v>
       </c>
-      <c r="T1" s="9" t="s">
+      <c r="U1" s="9" t="s">
         <v>17</v>
       </c>
-      <c r="U1" s="9" t="s">
+      <c r="V1" s="9" t="s">
         <v>18</v>
       </c>
-      <c r="V1" s="9" t="s">
+      <c r="W1" s="9" t="s">
         <v>19</v>
       </c>
-      <c r="W1" s="9" t="s">
+      <c r="X1" s="9" t="s">
         <v>20</v>
-      </c>
-      <c r="X1" s="9" t="s">
-        <v>21</v>
       </c>
     </row>
     <row r="2" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A2" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="B2" s="10" t="s">
         <v>22</v>
-      </c>
-      <c r="B2" s="10" t="s">
-        <v>23</v>
       </c>
       <c r="C2" s="11">
         <v>800</v>
@@ -644,14 +647,14 @@
       <c r="D2" s="4">
         <v>0.9</v>
       </c>
-      <c r="E2" s="4">
-        <v>51</v>
+      <c r="E2" s="4" t="s">
+        <v>26</v>
       </c>
       <c r="F2" s="4">
         <v>7</v>
       </c>
       <c r="G2" s="2">
-        <v>65</v>
+        <v>60</v>
       </c>
       <c r="H2" s="2">
         <v>7.9</v>

</xml_diff>